<commit_message>
updating region data file
</commit_message>
<xml_diff>
--- a/Region_data.xlsx
+++ b/Region_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\githubs\contact_wire_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8372ADEF-D2CF-4082-840D-0EB2DB92683A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2CCF52C-BCED-4D9D-83AC-EAFF38DA1361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3645" yWindow="1425" windowWidth="21195" windowHeight="13020" activeTab="4" xr2:uid="{62DB6618-FD48-415E-A163-826BF443D327}"/>
+    <workbookView xWindow="32925" yWindow="1500" windowWidth="21195" windowHeight="13020" activeTab="4" xr2:uid="{62DB6618-FD48-415E-A163-826BF443D327}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="91">
   <si>
     <t>neutral section names</t>
   </si>
@@ -260,72 +260,21 @@
     <t>Asset_Number</t>
   </si>
   <si>
-    <t>Second_Name</t>
-  </si>
-  <si>
     <t>Sentinal</t>
   </si>
   <si>
     <t>Level</t>
   </si>
   <si>
-    <t>Jim</t>
-  </si>
-  <si>
-    <t>Evans</t>
-  </si>
-  <si>
     <t>PW</t>
   </si>
   <si>
-    <t>dh</t>
-  </si>
-  <si>
-    <t>Mark</t>
-  </si>
-  <si>
-    <t>Kevin</t>
-  </si>
-  <si>
-    <t>Hetherington</t>
-  </si>
-  <si>
     <t>kh</t>
   </si>
   <si>
-    <t>Charlotte</t>
-  </si>
-  <si>
-    <t>Barrett</t>
-  </si>
-  <si>
     <t>cb</t>
   </si>
   <si>
-    <t>Hamilton</t>
-  </si>
-  <si>
-    <t>Karl</t>
-  </si>
-  <si>
-    <t>Luke</t>
-  </si>
-  <si>
-    <t>Scott</t>
-  </si>
-  <si>
-    <t>Sarah</t>
-  </si>
-  <si>
-    <t>Bar</t>
-  </si>
-  <si>
-    <t>Terance</t>
-  </si>
-  <si>
-    <t>Brown</t>
-  </si>
-  <si>
     <t>ls</t>
   </si>
   <si>
@@ -335,7 +284,25 @@
     <t>tb</t>
   </si>
   <si>
-    <t>First_Name</t>
+    <t>Kevin Hetherington</t>
+  </si>
+  <si>
+    <t>Charlotte Barrett</t>
+  </si>
+  <si>
+    <t>Karl Hamilton</t>
+  </si>
+  <si>
+    <t>Luke Scott</t>
+  </si>
+  <si>
+    <t>Sarah Bar</t>
+  </si>
+  <si>
+    <t>Terance Brown</t>
+  </si>
+  <si>
+    <t>Name</t>
   </si>
 </sst>
 </file>
@@ -1582,17 +1549,16 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8969DD6-61AF-495A-B637-779D81187039}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="B1" t="s">
         <v>76</v>
@@ -1603,144 +1569,89 @@
       <c r="D1" t="s">
         <v>78</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2">
+        <v>74157</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
         <v>79</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3">
+        <v>141012</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
         <v>80</v>
       </c>
-      <c r="C2">
-        <v>140968</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3">
-        <v>150270</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
-      </c>
-      <c r="B4" t="s">
-        <v>85</v>
+        <v>86</v>
+      </c>
+      <c r="B4">
+        <v>116105</v>
       </c>
       <c r="C4">
-        <v>74157</v>
-      </c>
-      <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>87</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5">
+        <v>143208</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>88</v>
       </c>
-      <c r="C5">
-        <v>141012</v>
-      </c>
-      <c r="D5">
+      <c r="B6">
+        <v>1111595</v>
+      </c>
+      <c r="C6">
         <v>1</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>91</v>
-      </c>
-      <c r="B6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C6">
-        <v>116105</v>
-      </c>
-      <c r="D6">
+      <c r="B7">
+        <v>1259055</v>
+      </c>
+      <c r="C7">
         <v>1</v>
       </c>
-      <c r="E6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" t="s">
-        <v>93</v>
-      </c>
-      <c r="C7">
-        <v>143208</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>94</v>
-      </c>
-      <c r="B8" t="s">
-        <v>95</v>
-      </c>
-      <c r="C8">
-        <v>1111595</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B9" t="s">
-        <v>97</v>
-      </c>
-      <c r="C9">
-        <v>1259055</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
-        <v>100</v>
+      <c r="D7" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -2336,6 +2247,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="cb6380d2-b01f-4e04-9200-9666676ed141" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002A49252DC7531642B064D59214E738D4" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2e90bbfbf4f52bf4a6656f5589d033bb">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="cb6380d2-b01f-4e04-9200-9666676ed141" xmlns:ns4="f068c7d5-04e7-4821-88a1-b1f97a388bb7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d814bd8026fe29e70e1bc18c824ed2a7" ns3:_="" ns4:_="">
     <xsd:import namespace="cb6380d2-b01f-4e04-9200-9666676ed141"/>
@@ -2588,24 +2516,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06A62760-3B76-45B2-B7CB-74304B7ECF2A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="f068c7d5-04e7-4821-88a1-b1f97a388bb7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="cb6380d2-b01f-4e04-9200-9666676ed141"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="cb6380d2-b01f-4e04-9200-9666676ed141" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC417360-1F6A-4D75-9B30-CA996FA04E31}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6848DD44-78B0-4924-8517-B02B8138DA94}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2622,29 +2558,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC417360-1F6A-4D75-9B30-CA996FA04E31}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06A62760-3B76-45B2-B7CB-74304B7ECF2A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="f068c7d5-04e7-4821-88a1-b1f97a388bb7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="cb6380d2-b01f-4e04-9200-9666676ed141"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>